<commit_message>
Fix Apple label colors, add (x86)/(ARM) tags, tidy Outputs folder
Excel: remove 3 blank rows in Authors sheet so Test17 sits directly
after Test16 — fixes the off-by-one that caused the position-based
manufacturer lookup to return None for Test17.

Notebook (both heatmap and barchart functions): replace fragile
col_idx-1 position lookup with an ID-based lookup (extra_meta_data['#']
== 'TestN'). Appends ' (ARM)' or ' (x86)' to every series label using
the new 'Exe Architecture' column — heatmap y-axis labels and legend
entries now clearly distinguish the two exe types. Apple M5 (ARM) row
correctly renders in blue.

Outputs: move superseded plots to old_plots/ (gitignored); keep only
the current run. Copy exe_comparison_WorkM5 to images/ and add it to
the README new-findings section.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Runtimes/ByscayneMode_Benchmarks.xlsx
+++ b/Runtimes/ByscayneMode_Benchmarks.xlsx
@@ -2134,7 +2134,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="31.1640625" customWidth="1" min="2" max="2"/>
@@ -3095,71 +3095,60 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="57" t="n"/>
-      <c r="D18" s="57" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="57" t="n"/>
-      <c r="D19" s="57" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="57" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Test17</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>roh@sgmco.cl</t>
         </is>
       </c>
-      <c r="C21" s="60" t="n">
+      <c r="C18" s="60" t="n">
         <v>46119</v>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>macOS</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>M5</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>WorkM5</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>(10c-4.61GHz)</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>ARM64 (gfortran)</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>Apple</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>MacBook Pro Laptop</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>Native ARM64; usgt_180_arm compiled with gfortran via Homebrew GCC</t>
         </is>

</xml_diff>

<commit_message>
Add WorkM3 (M3 Max) and SGM035 (M4) ARM results; new 1-to-1 M3 Max plot
Results database:
- Test18: WorkM3 M3 Max ARM64 (gfortran) — full 1–16 agent sweep
- Test19: SGM035 M4 ARM64 (gfortran) — partial (16-agent run only,
  submitted in old agent_runtimes format; full sweep pending)

Plots regenerated with updated dataset (19 tests + 1 partial):
- exe_comparison_WorkM3: new 1-to-1 comparison M3 Max x86 vs ARM native
- exe_comparison_WorkM5: refreshed with latest data
- runtime_heatmap, runtime_statistics, runtime_best_lineplot: all updated

README: add M3 Max comparison figure; note M4 1-to-1 pending full sweep.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Runtimes/ByscayneMode_Benchmarks.xlsx
+++ b/Runtimes/ByscayneMode_Benchmarks.xlsx
@@ -839,7 +839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R20"/>
+  <dimension ref="A1:T20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12"/>
   <cols>
     <col width="12.1640625" customWidth="1" style="2" min="1" max="1"/>
@@ -952,6 +952,16 @@
           <t>M5</t>
         </is>
       </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>M3 Max</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -1044,6 +1054,16 @@
           <t>WorkM5</t>
         </is>
       </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>WorkM3</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>SGM035</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14" customHeight="1">
       <c r="A3" s="31" t="inlineStr">
@@ -1136,6 +1156,16 @@
           <t>(10c-4.61GHz)</t>
         </is>
       </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>(16c-4.05 GHz)</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>(10c-4.51 GHz)</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="13" customHeight="1">
       <c r="A4" s="47" t="inlineStr">
@@ -1226,6 +1256,16 @@
       <c r="R4" t="inlineStr">
         <is>
           <t>Test17</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Test18</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Test19</t>
         </is>
       </c>
     </row>
@@ -1284,6 +1324,9 @@
       <c r="R5" t="n">
         <v>3.478</v>
       </c>
+      <c r="S5" t="n">
+        <v>4.7354</v>
+      </c>
     </row>
     <row r="6" customFormat="1" s="54">
       <c r="A6" s="17" t="n">
@@ -1340,6 +1383,9 @@
       <c r="R6" t="n">
         <v>3.7012</v>
       </c>
+      <c r="S6" t="n">
+        <v>4.7135</v>
+      </c>
     </row>
     <row r="7" customFormat="1" s="54">
       <c r="A7" s="17" t="n">
@@ -1396,6 +1442,9 @@
       <c r="R7" t="n">
         <v>3.9802</v>
       </c>
+      <c r="S7" t="n">
+        <v>4.7988</v>
+      </c>
     </row>
     <row r="8" customFormat="1" s="54">
       <c r="A8" s="17" t="n">
@@ -1452,6 +1501,9 @@
       <c r="R8" t="n">
         <v>4.3041</v>
       </c>
+      <c r="S8" t="n">
+        <v>4.7793</v>
+      </c>
     </row>
     <row r="9" customFormat="1" s="54">
       <c r="A9" s="17" t="n">
@@ -1508,6 +1560,9 @@
       <c r="R9" t="n">
         <v>4.636</v>
       </c>
+      <c r="S9" t="n">
+        <v>4.7951</v>
+      </c>
     </row>
     <row r="10" customFormat="1" s="54">
       <c r="A10" s="17" t="n">
@@ -1562,6 +1617,9 @@
       <c r="R10" t="n">
         <v>5.016</v>
       </c>
+      <c r="S10" t="n">
+        <v>4.8687</v>
+      </c>
     </row>
     <row r="11" customFormat="1" s="54">
       <c r="A11" s="18" t="n">
@@ -1618,6 +1676,9 @@
       <c r="R11" t="n">
         <v>5.4074</v>
       </c>
+      <c r="S11" t="n">
+        <v>5.0869</v>
+      </c>
     </row>
     <row r="12" customFormat="1" s="54">
       <c r="A12" s="17" t="n">
@@ -1674,6 +1735,9 @@
       <c r="R12" t="n">
         <v>5.6641</v>
       </c>
+      <c r="S12" t="n">
+        <v>5.2382</v>
+      </c>
     </row>
     <row r="13" customFormat="1" s="54">
       <c r="A13" s="17" t="n">
@@ -1728,6 +1792,9 @@
       <c r="R13" t="n">
         <v>6.2495</v>
       </c>
+      <c r="S13" t="n">
+        <v>5.8334</v>
+      </c>
     </row>
     <row r="14" customFormat="1" s="54">
       <c r="A14" s="17" t="n">
@@ -1782,6 +1849,9 @@
       <c r="R14" t="n">
         <v>6.8451</v>
       </c>
+      <c r="S14" t="n">
+        <v>6.321</v>
+      </c>
     </row>
     <row r="15" customFormat="1" s="54">
       <c r="A15" s="17" t="n">
@@ -1839,6 +1909,9 @@
       <c r="R15" t="n">
         <v>7.7447</v>
       </c>
+      <c r="S15" t="n">
+        <v>7.181</v>
+      </c>
     </row>
     <row r="16" customFormat="1" s="54">
       <c r="A16" s="17" t="n">
@@ -1896,6 +1969,9 @@
       <c r="R16" t="n">
         <v>8.3064</v>
       </c>
+      <c r="S16" t="n">
+        <v>7.6501</v>
+      </c>
     </row>
     <row r="17" customFormat="1" s="54">
       <c r="A17" s="17" t="n">
@@ -1951,6 +2027,9 @@
       <c r="R17" t="n">
         <v>9.1073</v>
       </c>
+      <c r="S17" t="n">
+        <v>8.379799999999999</v>
+      </c>
     </row>
     <row r="18" customFormat="1" s="54">
       <c r="A18" s="17" t="n">
@@ -2008,6 +2087,9 @@
       <c r="R18" t="n">
         <v>9.8291</v>
       </c>
+      <c r="S18" t="n">
+        <v>9.0161</v>
+      </c>
     </row>
     <row r="19" customFormat="1" s="54">
       <c r="A19" s="17" t="n">
@@ -2065,6 +2147,9 @@
       <c r="R19" t="n">
         <v>10.8483</v>
       </c>
+      <c r="S19" t="n">
+        <v>9.616099999999999</v>
+      </c>
     </row>
     <row r="20" customFormat="1" s="54">
       <c r="A20" s="17" t="n">
@@ -2120,6 +2205,12 @@
       </c>
       <c r="R20" t="n">
         <v>11.3681</v>
+      </c>
+      <c r="S20" t="n">
+        <v>10.1899</v>
+      </c>
+      <c r="T20" t="n">
+        <v>13.6628</v>
       </c>
     </row>
   </sheetData>
@@ -2134,7 +2225,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="31.1640625" customWidth="1" min="2" max="2"/>
@@ -3151,6 +3242,126 @@
       <c r="L18" t="inlineStr">
         <is>
           <t>Native ARM64; usgt_180_arm compiled with gfortran via Homebrew GCC</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Test18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>roh@sgmco.cl</t>
+        </is>
+      </c>
+      <c r="C19" s="60" t="n">
+        <v>46129</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>macOS</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>M3 Max</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>WorkM3</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>(16c-4.05 GHz)</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>ARM64 (gfortran)</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>MacBook Pro Laptop</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Native ARM64; usgt_180_arm</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Test19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>roh@sgmco.cl</t>
+        </is>
+      </c>
+      <c r="C20" s="60" t="n">
+        <v>46129</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>macOS</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>SGM035</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>(10c-4.51 GHz)</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>ARM64 (gfortran)</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Mac Mini</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Partial — 16-agent run only (old agent_runtimes format); full sweep pending</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Test19 (SGM035 M4 ARM) full 1-16 agent sweep
- Excel: Test19 col 20 populated with complete 1-16 runtimes (3.60–13.66 min)
  from SGM035_2026-04-17_142100_benchmark_results_new.csv (replaces 16-agent-only partial data)
- Notebook re-executed: heatmap and statistics updated with full SGM035 ARM data
- images/: updated runtime_heatmap.png and runtime_statistics.png
- README: removed "M4 1-to-1 pending" note; clarified that a paired
  exe comparison requires an x86 run on SGM035 specifically (existing M4 x86
  is SGM023, a different unit)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Runtimes/ByscayneMode_Benchmarks.xlsx
+++ b/Runtimes/ByscayneMode_Benchmarks.xlsx
@@ -1327,6 +1327,9 @@
       <c r="S5" t="n">
         <v>4.7354</v>
       </c>
+      <c r="T5" t="n">
+        <v>3.6019</v>
+      </c>
     </row>
     <row r="6" customFormat="1" s="54">
       <c r="A6" s="17" t="n">
@@ -1386,6 +1389,9 @@
       <c r="S6" t="n">
         <v>4.7135</v>
       </c>
+      <c r="T6" t="n">
+        <v>3.9379</v>
+      </c>
     </row>
     <row r="7" customFormat="1" s="54">
       <c r="A7" s="17" t="n">
@@ -1445,6 +1451,9 @@
       <c r="S7" t="n">
         <v>4.7988</v>
       </c>
+      <c r="T7" t="n">
+        <v>4.128</v>
+      </c>
     </row>
     <row r="8" customFormat="1" s="54">
       <c r="A8" s="17" t="n">
@@ -1504,6 +1513,9 @@
       <c r="S8" t="n">
         <v>4.7793</v>
       </c>
+      <c r="T8" t="n">
+        <v>4.5206</v>
+      </c>
     </row>
     <row r="9" customFormat="1" s="54">
       <c r="A9" s="17" t="n">
@@ -1563,6 +1575,9 @@
       <c r="S9" t="n">
         <v>4.7951</v>
       </c>
+      <c r="T9" t="n">
+        <v>5.052</v>
+      </c>
     </row>
     <row r="10" customFormat="1" s="54">
       <c r="A10" s="17" t="n">
@@ -1620,6 +1635,9 @@
       <c r="S10" t="n">
         <v>4.8687</v>
       </c>
+      <c r="T10" t="n">
+        <v>5.5552</v>
+      </c>
     </row>
     <row r="11" customFormat="1" s="54">
       <c r="A11" s="18" t="n">
@@ -1679,6 +1697,9 @@
       <c r="S11" t="n">
         <v>5.0869</v>
       </c>
+      <c r="T11" t="n">
+        <v>6.1346</v>
+      </c>
     </row>
     <row r="12" customFormat="1" s="54">
       <c r="A12" s="17" t="n">
@@ -1738,6 +1759,9 @@
       <c r="S12" t="n">
         <v>5.2382</v>
       </c>
+      <c r="T12" t="n">
+        <v>6.8325</v>
+      </c>
     </row>
     <row r="13" customFormat="1" s="54">
       <c r="A13" s="17" t="n">
@@ -1795,6 +1819,9 @@
       <c r="S13" t="n">
         <v>5.8334</v>
       </c>
+      <c r="T13" t="n">
+        <v>7.5822</v>
+      </c>
     </row>
     <row r="14" customFormat="1" s="54">
       <c r="A14" s="17" t="n">
@@ -1852,6 +1879,9 @@
       <c r="S14" t="n">
         <v>6.321</v>
       </c>
+      <c r="T14" t="n">
+        <v>8.4147</v>
+      </c>
     </row>
     <row r="15" customFormat="1" s="54">
       <c r="A15" s="17" t="n">
@@ -1912,6 +1942,9 @@
       <c r="S15" t="n">
         <v>7.181</v>
       </c>
+      <c r="T15" t="n">
+        <v>9.288600000000001</v>
+      </c>
     </row>
     <row r="16" customFormat="1" s="54">
       <c r="A16" s="17" t="n">
@@ -1972,6 +2005,9 @@
       <c r="S16" t="n">
         <v>7.6501</v>
       </c>
+      <c r="T16" t="n">
+        <v>10.1908</v>
+      </c>
     </row>
     <row r="17" customFormat="1" s="54">
       <c r="A17" s="17" t="n">
@@ -2030,6 +2066,9 @@
       <c r="S17" t="n">
         <v>8.379799999999999</v>
       </c>
+      <c r="T17" t="n">
+        <v>11.0448</v>
+      </c>
     </row>
     <row r="18" customFormat="1" s="54">
       <c r="A18" s="17" t="n">
@@ -2090,6 +2129,9 @@
       <c r="S18" t="n">
         <v>9.0161</v>
       </c>
+      <c r="T18" t="n">
+        <v>11.9249</v>
+      </c>
     </row>
     <row r="19" customFormat="1" s="54">
       <c r="A19" s="17" t="n">
@@ -2149,6 +2191,9 @@
       </c>
       <c r="S19" t="n">
         <v>9.616099999999999</v>
+      </c>
+      <c r="T19" t="n">
+        <v>12.7899</v>
       </c>
     </row>
     <row r="20" customFormat="1" s="54">
@@ -3361,7 +3406,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Partial — 16-agent run only (old agent_runtimes format); full sweep pending</t>
+          <t>Native ARM64; usgt_180_arm compiled with gfortran via Homebrew GCC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add SGM001 M1 exe comparison plot; fix trailing spaces in Author names
- Excel: fixed trailing spaces in Computer names (SGM001, SGM005, ESI)
  — had prevented SGM001 from being auto-discovered as a paired machine
- Notebook re-executed: SGM001 x86 vs ARM comparison now auto-generated
  (1.20x speedup, 16% shorter mean runtime; steep 5x slope 1→16 agents)
- images/: exe_comparison_SGM001.png added; heatmap, statistics, lineplot updated
- README: SGM001 plot embedded with M1 thermal behaviour note explaining
  the steep agent-count slope vs the near-flat M4/M5 curves

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Runtimes/ByscayneMode_Benchmarks.xlsx
+++ b/Runtimes/ByscayneMode_Benchmarks.xlsx
@@ -2878,7 +2878,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">SGM001 </t>
+          <t>SGM001</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -2938,7 +2938,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve">SGM005 </t>
+          <t>SGM005</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -3419,7 +3419,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t xml:space="preserve">ESI </t>
+          <t>ESI</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">

</xml_diff>

<commit_message>
Add Test22 (WorkM2 M2 Pro ARM native); note SGM005 M2 run in progress
- Excel: Test22 — WorkM2, Apple M2 Pro, ARM64 gfortran, automated script
  (runtimes 4.92–10.21 min, 1–16 agents; mean 6.71 min)
- Notebook re-executed: WorkM2 comparison auto-generated (1.24x, 20% shorter)
  — paired machines now: SGM001, WorkM2, WorkM3, WorkM5
- images/: exe_comparison_WorkM2.png added; all plots updated
- README: WorkM2 plot embedded; SGM005 M2 noted as in progress

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Runtimes/ByscayneMode_Benchmarks.xlsx
+++ b/Runtimes/ByscayneMode_Benchmarks.xlsx
@@ -841,7 +841,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V20"/>
+  <dimension ref="A1:W20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12"/>
   <cols>
     <col width="12.1640625" customWidth="1" style="2" min="1" max="1"/>
@@ -974,6 +974,11 @@
           <t>M1</t>
         </is>
       </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>M2 Pro</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -1086,6 +1091,11 @@
           <t>SGM001</t>
         </is>
       </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>WorkM2</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14" customHeight="1">
       <c r="A3" s="31" t="inlineStr">
@@ -1198,6 +1208,11 @@
           <t>(8c-3.2 GHz)</t>
         </is>
       </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>(12c-3.48GHz)</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="13" customHeight="1">
       <c r="A4" s="47" t="inlineStr">
@@ -1308,6 +1323,11 @@
       <c r="V4" t="inlineStr">
         <is>
           <t>Test21</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Test22</t>
         </is>
       </c>
     </row>
@@ -1378,6 +1398,9 @@
       <c r="V5" t="n">
         <v>5.099933</v>
       </c>
+      <c r="W5" t="n">
+        <v>4.9245</v>
+      </c>
     </row>
     <row r="6" customFormat="1" s="54">
       <c r="A6" s="17" t="n">
@@ -1446,6 +1469,9 @@
       <c r="V6" t="n">
         <v>5.389</v>
       </c>
+      <c r="W6" t="n">
+        <v>5.012633</v>
+      </c>
     </row>
     <row r="7" customFormat="1" s="54">
       <c r="A7" s="17" t="n">
@@ -1514,6 +1540,9 @@
       <c r="V7" t="n">
         <v>5.755717</v>
       </c>
+      <c r="W7" t="n">
+        <v>5.111433</v>
+      </c>
     </row>
     <row r="8" customFormat="1" s="54">
       <c r="A8" s="17" t="n">
@@ -1582,6 +1611,9 @@
       <c r="V8" t="n">
         <v>6.399867</v>
       </c>
+      <c r="W8" t="n">
+        <v>5.1694</v>
+      </c>
     </row>
     <row r="9" customFormat="1" s="54">
       <c r="A9" s="17" t="n">
@@ -1650,6 +1682,9 @@
       <c r="V9" t="n">
         <v>7.730017</v>
       </c>
+      <c r="W9" t="n">
+        <v>5.35155</v>
+      </c>
     </row>
     <row r="10" customFormat="1" s="54">
       <c r="A10" s="17" t="n">
@@ -1716,6 +1751,9 @@
       <c r="V10" t="n">
         <v>9.249582999999999</v>
       </c>
+      <c r="W10" t="n">
+        <v>5.435383</v>
+      </c>
     </row>
     <row r="11" customFormat="1" s="54">
       <c r="A11" s="18" t="n">
@@ -1784,6 +1822,9 @@
       <c r="V11" t="n">
         <v>10.87425</v>
       </c>
+      <c r="W11" t="n">
+        <v>5.867167</v>
+      </c>
     </row>
     <row r="12" customFormat="1" s="54">
       <c r="A12" s="17" t="n">
@@ -1852,6 +1893,9 @@
       <c r="V12" t="n">
         <v>12.552017</v>
       </c>
+      <c r="W12" t="n">
+        <v>5.773</v>
+      </c>
     </row>
     <row r="13" customFormat="1" s="54">
       <c r="A13" s="17" t="n">
@@ -1918,6 +1962,9 @@
       <c r="V13" t="n">
         <v>14.174833</v>
       </c>
+      <c r="W13" t="n">
+        <v>6.203467</v>
+      </c>
     </row>
     <row r="14" customFormat="1" s="54">
       <c r="A14" s="17" t="n">
@@ -1984,6 +2031,9 @@
       <c r="V14" t="n">
         <v>15.798233</v>
       </c>
+      <c r="W14" t="n">
+        <v>6.63255</v>
+      </c>
     </row>
     <row r="15" customFormat="1" s="54">
       <c r="A15" s="17" t="n">
@@ -2053,6 +2103,9 @@
       <c r="V15" t="n">
         <v>17.43005</v>
       </c>
+      <c r="W15" t="n">
+        <v>7.125233</v>
+      </c>
     </row>
     <row r="16" customFormat="1" s="54">
       <c r="A16" s="17" t="n">
@@ -2122,6 +2175,9 @@
       <c r="V16" t="n">
         <v>19.028917</v>
       </c>
+      <c r="W16" t="n">
+        <v>7.5704</v>
+      </c>
     </row>
     <row r="17" customFormat="1" s="54">
       <c r="A17" s="17" t="n">
@@ -2189,6 +2245,9 @@
       <c r="V17" t="n">
         <v>20.642117</v>
       </c>
+      <c r="W17" t="n">
+        <v>8.410717</v>
+      </c>
     </row>
     <row r="18" customFormat="1" s="54">
       <c r="A18" s="17" t="n">
@@ -2258,6 +2317,9 @@
       <c r="V18" t="n">
         <v>22.246817</v>
       </c>
+      <c r="W18" t="n">
+        <v>9.02685</v>
+      </c>
     </row>
     <row r="19" customFormat="1" s="54">
       <c r="A19" s="17" t="n">
@@ -2327,6 +2389,9 @@
       <c r="V19" t="n">
         <v>23.87075</v>
       </c>
+      <c r="W19" t="n">
+        <v>9.576333</v>
+      </c>
     </row>
     <row r="20" customFormat="1" s="54">
       <c r="A20" s="17" t="n">
@@ -2394,6 +2459,9 @@
       </c>
       <c r="V20" t="n">
         <v>25.506583</v>
+      </c>
+      <c r="W20" t="n">
+        <v>10.207567</v>
       </c>
     </row>
   </sheetData>
@@ -2408,7 +2476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M22"/>
+  <dimension ref="A1:M23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="31.1640625" customWidth="1" min="2" max="2"/>
@@ -3773,6 +3841,71 @@
         </is>
       </c>
       <c r="M22" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Test22</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>roh@sgmco.cl</t>
+        </is>
+      </c>
+      <c r="C23" s="61" t="n">
+        <v>46132</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>macOS</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>M2 Pro</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>WorkM2</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>(12c-3.48GHz)</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>ARM64 (gfortran)</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>MacBook Pro Laptop</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Native ARM64; usgt_180_arm; automated script</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
         <is>
           <t>automated</t>
         </is>

</xml_diff>

<commit_message>
Add Test23 (SGM005 M2 ARM native); five machines now have paired exe comparisons
- Excel: Test23 — SGM005, Apple M2, ARM64 gfortran, automated script
  (runtimes 4.80–20.97 min; mean 11.60 min vs x86 mean 12.88 min)
- Notebook re-executed: SGM005 comparison auto-generated (1.11x, 10% shorter)
  Paired machines: SGM001 (M1), SGM005 (M2), WorkM2 (M2 Pro),
                   WorkM3 (M3 Max), WorkM5 (M5)
- images/: exe_comparison_SGM005.png added; all plots updated
- README: SGM005 plot embedded with M2 thermal note; in-progress notice removed

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Runtimes/ByscayneMode_Benchmarks.xlsx
+++ b/Runtimes/ByscayneMode_Benchmarks.xlsx
@@ -841,7 +841,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W20"/>
+  <dimension ref="A1:X20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12"/>
   <cols>
     <col width="12.1640625" customWidth="1" style="2" min="1" max="1"/>
@@ -979,6 +979,11 @@
           <t>M2 Pro</t>
         </is>
       </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -1096,6 +1101,11 @@
           <t>WorkM2</t>
         </is>
       </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>SGM005</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14" customHeight="1">
       <c r="A3" s="31" t="inlineStr">
@@ -1213,6 +1223,11 @@
           <t>(12c-3.48GHz)</t>
         </is>
       </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>(8c-3.49 GHz)</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="13" customHeight="1">
       <c r="A4" s="47" t="inlineStr">
@@ -1328,6 +1343,11 @@
       <c r="W4" t="inlineStr">
         <is>
           <t>Test22</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>Test23</t>
         </is>
       </c>
     </row>
@@ -1401,6 +1421,9 @@
       <c r="W5" t="n">
         <v>4.9245</v>
       </c>
+      <c r="X5" t="n">
+        <v>4.79765</v>
+      </c>
     </row>
     <row r="6" customFormat="1" s="54">
       <c r="A6" s="17" t="n">
@@ -1472,6 +1495,9 @@
       <c r="W6" t="n">
         <v>5.012633</v>
       </c>
+      <c r="X6" t="n">
+        <v>5.149467</v>
+      </c>
     </row>
     <row r="7" customFormat="1" s="54">
       <c r="A7" s="17" t="n">
@@ -1543,6 +1569,9 @@
       <c r="W7" t="n">
         <v>5.111433</v>
       </c>
+      <c r="X7" t="n">
+        <v>5.50225</v>
+      </c>
     </row>
     <row r="8" customFormat="1" s="54">
       <c r="A8" s="17" t="n">
@@ -1614,6 +1643,9 @@
       <c r="W8" t="n">
         <v>5.1694</v>
       </c>
+      <c r="X8" t="n">
+        <v>5.8126</v>
+      </c>
     </row>
     <row r="9" customFormat="1" s="54">
       <c r="A9" s="17" t="n">
@@ -1685,6 +1717,9 @@
       <c r="W9" t="n">
         <v>5.35155</v>
       </c>
+      <c r="X9" t="n">
+        <v>6.67115</v>
+      </c>
     </row>
     <row r="10" customFormat="1" s="54">
       <c r="A10" s="17" t="n">
@@ -1754,6 +1789,9 @@
       <c r="W10" t="n">
         <v>5.435383</v>
       </c>
+      <c r="X10" t="n">
+        <v>7.699667</v>
+      </c>
     </row>
     <row r="11" customFormat="1" s="54">
       <c r="A11" s="18" t="n">
@@ -1825,6 +1863,9 @@
       <c r="W11" t="n">
         <v>5.867167</v>
       </c>
+      <c r="X11" t="n">
+        <v>8.978717</v>
+      </c>
     </row>
     <row r="12" customFormat="1" s="54">
       <c r="A12" s="17" t="n">
@@ -1896,6 +1937,9 @@
       <c r="W12" t="n">
         <v>5.773</v>
       </c>
+      <c r="X12" t="n">
+        <v>10.343867</v>
+      </c>
     </row>
     <row r="13" customFormat="1" s="54">
       <c r="A13" s="17" t="n">
@@ -1965,6 +2009,9 @@
       <c r="W13" t="n">
         <v>6.203467</v>
       </c>
+      <c r="X13" t="n">
+        <v>11.649117</v>
+      </c>
     </row>
     <row r="14" customFormat="1" s="54">
       <c r="A14" s="17" t="n">
@@ -2034,6 +2081,9 @@
       <c r="W14" t="n">
         <v>6.63255</v>
       </c>
+      <c r="X14" t="n">
+        <v>13.0017</v>
+      </c>
     </row>
     <row r="15" customFormat="1" s="54">
       <c r="A15" s="17" t="n">
@@ -2106,6 +2156,9 @@
       <c r="W15" t="n">
         <v>7.125233</v>
       </c>
+      <c r="X15" t="n">
+        <v>14.335783</v>
+      </c>
     </row>
     <row r="16" customFormat="1" s="54">
       <c r="A16" s="17" t="n">
@@ -2178,6 +2231,9 @@
       <c r="W16" t="n">
         <v>7.5704</v>
       </c>
+      <c r="X16" t="n">
+        <v>15.682383</v>
+      </c>
     </row>
     <row r="17" customFormat="1" s="54">
       <c r="A17" s="17" t="n">
@@ -2248,6 +2304,9 @@
       <c r="W17" t="n">
         <v>8.410717</v>
       </c>
+      <c r="X17" t="n">
+        <v>17.007183</v>
+      </c>
     </row>
     <row r="18" customFormat="1" s="54">
       <c r="A18" s="17" t="n">
@@ -2320,6 +2379,9 @@
       <c r="W18" t="n">
         <v>9.02685</v>
       </c>
+      <c r="X18" t="n">
+        <v>18.312267</v>
+      </c>
     </row>
     <row r="19" customFormat="1" s="54">
       <c r="A19" s="17" t="n">
@@ -2392,6 +2454,9 @@
       <c r="W19" t="n">
         <v>9.576333</v>
       </c>
+      <c r="X19" t="n">
+        <v>19.64135</v>
+      </c>
     </row>
     <row r="20" customFormat="1" s="54">
       <c r="A20" s="17" t="n">
@@ -2462,6 +2527,9 @@
       </c>
       <c r="W20" t="n">
         <v>10.207567</v>
+      </c>
+      <c r="X20" t="n">
+        <v>20.973967</v>
       </c>
     </row>
   </sheetData>
@@ -2476,7 +2544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:M24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="31.1640625" customWidth="1" min="2" max="2"/>
@@ -3906,6 +3974,71 @@
         </is>
       </c>
       <c r="M23" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Test23</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>roh@sgmco.cl</t>
+        </is>
+      </c>
+      <c r="C24" s="61" t="n">
+        <v>46132</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>macOS</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>SGM005</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>(8c-3.49 GHz)</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>ARM64 (gfortran)</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Mac Mini</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Native ARM64; usgt_180_arm; automated script</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
         <is>
           <t>automated</t>
         </is>

</xml_diff>